<commit_message>
se adjunto la ultima actualizacion del projecto TestGateway
</commit_message>
<xml_diff>
--- a/src/main/java/Data/Import.xlsx
+++ b/src/main/java/Data/Import.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bdsyc\OneDrive\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073EB9B5-7AB7-42F6-9675-EA0554EE18C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B37B51-5520-440A-9F02-20BC6583B71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Banco a Banco" sheetId="2" r:id="rId1"/>
     <sheet name="Bancos externos" sheetId="1" r:id="rId2"/>
+    <sheet name="Domiciliacion" sheetId="3" r:id="rId3"/>
+    <sheet name="DTA" sheetId="4" r:id="rId4"/>
+    <sheet name="IBPs" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="113">
   <si>
     <t>id</t>
   </si>
@@ -49,12 +52,6 @@
     <t>0114</t>
   </si>
   <si>
-    <t>Cliente Bancaribe Juridico</t>
-  </si>
-  <si>
-    <t>01140172461720020412</t>
-  </si>
-  <si>
     <t>V13951863</t>
   </si>
   <si>
@@ -82,9 +79,6 @@
     <t>Cliente BanPlus Juridico</t>
   </si>
   <si>
-    <t>J300558053</t>
-  </si>
-  <si>
     <t>Cliente de Venezolano de Crédito</t>
   </si>
   <si>
@@ -106,53 +100,292 @@
     <t>01740131991314182989</t>
   </si>
   <si>
-    <t>Ana Alvarez</t>
-  </si>
-  <si>
-    <t>CARRILLO DANGOND</t>
-  </si>
-  <si>
-    <t>P305884</t>
-  </si>
-  <si>
-    <t>01140190291900021336</t>
-  </si>
-  <si>
     <t>E84549121</t>
   </si>
   <si>
-    <t>LEON RIVERA</t>
-  </si>
-  <si>
     <t>01140165171659176870</t>
   </si>
   <si>
-    <t>G200161370</t>
-  </si>
-  <si>
-    <t>TELECOMUNICACIONES MOVILNET</t>
-  </si>
-  <si>
-    <t>01140150341500390600</t>
-  </si>
-  <si>
-    <t>CONSEJO COMUNAL</t>
-  </si>
-  <si>
-    <t>C310654948</t>
-  </si>
-  <si>
-    <t>01140184841840052555</t>
+    <t>email</t>
+  </si>
+  <si>
+    <t>abrahamescalona84@gmail.com</t>
+  </si>
+  <si>
+    <t>celeOTP</t>
+  </si>
+  <si>
+    <t>4129854529</t>
+  </si>
+  <si>
+    <t>04129854529</t>
+  </si>
+  <si>
+    <t>C200852369</t>
+  </si>
+  <si>
+    <t>R149985332</t>
+  </si>
+  <si>
+    <t>V10010700</t>
+  </si>
+  <si>
+    <t>V12571984</t>
+  </si>
+  <si>
+    <t>V14019712</t>
+  </si>
+  <si>
+    <t>J304248814</t>
+  </si>
+  <si>
+    <t>J307243287</t>
+  </si>
+  <si>
+    <t>0138</t>
+  </si>
+  <si>
+    <t>0108</t>
+  </si>
+  <si>
+    <t>0128</t>
+  </si>
+  <si>
+    <t>0105</t>
+  </si>
+  <si>
+    <t>04142157763</t>
+  </si>
+  <si>
+    <t>04242221350</t>
+  </si>
+  <si>
+    <t>04141876830</t>
+  </si>
+  <si>
+    <t>04241220315</t>
+  </si>
+  <si>
+    <t>04148989781</t>
+  </si>
+  <si>
+    <t>04241271948</t>
+  </si>
+  <si>
+    <t>Cliente Banplus</t>
+  </si>
+  <si>
+    <t>Cliente Plaza</t>
+  </si>
+  <si>
+    <t>Cliente Provincial</t>
+  </si>
+  <si>
+    <t>Cliente Caroni</t>
+  </si>
+  <si>
+    <t>Cliente Mercantil</t>
+  </si>
+  <si>
+    <t>J0000004</t>
+  </si>
+  <si>
+    <t>01740127111274200000</t>
+  </si>
+  <si>
+    <t>01740139441394130000</t>
+  </si>
+  <si>
+    <t>01080571600100080000</t>
+  </si>
+  <si>
+    <t>01280001190101010000</t>
+  </si>
+  <si>
+    <t>01050161071161020000</t>
+  </si>
+  <si>
+    <t>01280049584901990000</t>
+  </si>
+  <si>
+    <t>01380003190030160000</t>
+  </si>
+  <si>
+    <t>Ana Alvarez E</t>
+  </si>
+  <si>
+    <t>04125516274</t>
+  </si>
+  <si>
+    <t>J003439940</t>
+  </si>
+  <si>
+    <t>CARRILLO DANGOND J</t>
+  </si>
+  <si>
+    <t>Cliente Bancaribe v</t>
+  </si>
+  <si>
+    <t>04241747400</t>
+  </si>
+  <si>
+    <t>01140165111650173291</t>
+  </si>
+  <si>
+    <t>V18556186</t>
+  </si>
+  <si>
+    <t>01140164371640023739</t>
+  </si>
+  <si>
+    <t>LEON RIVERA J</t>
+  </si>
+  <si>
+    <t>01140164341640100393</t>
+  </si>
+  <si>
+    <t>04141861850</t>
+  </si>
+  <si>
+    <t>TELECOMUNICACIONES J</t>
+  </si>
+  <si>
+    <t>01140300043000118019</t>
+  </si>
+  <si>
+    <t>J085059148</t>
+  </si>
+  <si>
+    <t>Cliente J</t>
+  </si>
+  <si>
+    <t>01140223212230002730</t>
+  </si>
+  <si>
+    <t>J075768965</t>
+  </si>
+  <si>
+    <t>04124417813</t>
+  </si>
+  <si>
+    <t>01140521515210054601</t>
+  </si>
+  <si>
+    <t>04248263559</t>
+  </si>
+  <si>
+    <t>J303876056</t>
+  </si>
+  <si>
+    <t>J001091319</t>
+  </si>
+  <si>
+    <t>01140157111570019151</t>
+  </si>
+  <si>
+    <t>01140351463510043242</t>
+  </si>
+  <si>
+    <t>04143336175</t>
+  </si>
+  <si>
+    <t>04245226900</t>
+  </si>
+  <si>
+    <t>J300297381</t>
+  </si>
+  <si>
+    <t>Cliente Banplus C</t>
+  </si>
+  <si>
+    <t>01740127111274207669</t>
+  </si>
+  <si>
+    <t>01740139441394135873</t>
+  </si>
+  <si>
+    <t>01740130141304317074</t>
+  </si>
+  <si>
+    <t>J789456123</t>
+  </si>
+  <si>
+    <t>Cliente Banplus R</t>
+  </si>
+  <si>
+    <t>Cliente Banplus J</t>
+  </si>
+  <si>
+    <t>01380033250330007246</t>
+  </si>
+  <si>
+    <t>Plaza J</t>
+  </si>
+  <si>
+    <t>J00000202001</t>
+  </si>
+  <si>
+    <t>V00010010700</t>
+  </si>
+  <si>
+    <t>01380003190030161436</t>
+  </si>
+  <si>
+    <t>Plaza V</t>
+  </si>
+  <si>
+    <t>01080571600100084592</t>
+  </si>
+  <si>
+    <t>Provincial V</t>
+  </si>
+  <si>
+    <t>01280001190101015394</t>
+  </si>
+  <si>
+    <t>Cliente Caroni V</t>
+  </si>
+  <si>
+    <t>01280049584901992109</t>
+  </si>
+  <si>
+    <t>Cliente Caroni J</t>
+  </si>
+  <si>
+    <t>01050161071161022953</t>
+  </si>
+  <si>
+    <t>Cliente Mercantil J</t>
+  </si>
+  <si>
+    <t>01710002556002559050</t>
+  </si>
+  <si>
+    <t>Ciente Activo</t>
+  </si>
+  <si>
+    <t>0171</t>
+  </si>
+  <si>
+    <t>V24883412</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -175,14 +408,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -461,17 +697,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CF17BF3-6A57-46BE-A7DA-5B0694398C46}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1"/>
     <col min="2" max="2" width="30.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.5546875" style="1"/>
+    <col min="3" max="3" width="11.5546875" style="1"/>
+    <col min="4" max="4" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -488,126 +725,147 @@
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>62</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>69</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D5" s="1" t="s">
+        <v>78</v>
+      </c>
       <c r="E5" s="1" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D6" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="E6" s="1" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D7" s="1" t="s">
+        <v>85</v>
+      </c>
       <c r="E7" s="1" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D8" s="1" t="s">
+        <v>86</v>
+      </c>
       <c r="E8" s="1" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -617,17 +875,121 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1"/>
     <col min="2" max="2" width="28.5546875" style="1" customWidth="1"/>
-    <col min="3" max="4" width="11.5546875" style="1"/>
+    <col min="3" max="3" width="11.5546875" style="1"/>
+    <col min="4" max="4" width="12.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" style="1"/>
+    <col min="7" max="7" width="28.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.5546875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{013B165B-5FA5-4C9F-85A7-BF7729438ED5}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{8F1A32BA-8DE1-41AB-B188-3184BBF85AC7}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AC60F10-A41C-48DA-8C04-C602D7A2D831}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.5546875" style="1"/>
+    <col min="2" max="2" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1"/>
+    <col min="4" max="4" width="12.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,45 +1006,612 @@
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="E2" s="1" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>23</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D89D73B1-19E3-4D0A-9F8F-F0038872DEC5}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.5546875" style="1"/>
+    <col min="2" max="2" width="30.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1"/>
+    <col min="4" max="4" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="11.5546875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BE76DF0-6138-4991-9DEE-BC1774D8A5FD}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1"/>
+    <col min="4" max="4" width="12.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="11.5546875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>